<commit_message>
ADD csv version of categories dict
</commit_message>
<xml_diff>
--- a/output/leboncoin_catagories_with_id.xlsx
+++ b/output/leboncoin_catagories_with_id.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9707"/>
+    <workbookView windowWidth="23040" windowHeight="8987"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1931,7 +1931,7 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:B82" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A2:B82">
+    <sortState ref="A1:B82">
       <sortCondition ref="A1"/>
     </sortState>
     <extLst/>

</xml_diff>